<commit_message>
Updated with new codes and checks
</commit_message>
<xml_diff>
--- a/WGRDBESstockCoord/format/SCF/Example2_SCF_v2.xlsx
+++ b/WGRDBESstockCoord/format/SCF/Example2_SCF_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dtudk-my.sharepoint.com/personal/kibi_dtu_dk/Documents/RDBES_gits/RDBESstockCoord/WGRDBESstockCoord/format/SCF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="8_{D82F286C-0272-4FF6-8FFD-09EE9417A510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06512344-B90B-4E11-B2B0-D45CB5067048}"/>
+  <xr:revisionPtr revIDLastSave="151" documentId="8_{D82F286C-0272-4FF6-8FFD-09EE9417A510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BA92A5F-623B-483A-88EC-D782868CF11C}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{274BEBFC-7315-4E02-BADA-C86CAB5A4DD1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{274BEBFC-7315-4E02-BADA-C86CAB5A4DD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Catch (CC)" sheetId="1" r:id="rId1"/>
@@ -150,9 +150,6 @@
     <t>HAWG</t>
   </si>
   <si>
-    <t>HalfYear</t>
-  </si>
-  <si>
     <t>spr.27.3a4</t>
   </si>
   <si>
@@ -166,6 +163,9 @@
   </si>
   <si>
     <t>07-01</t>
+  </si>
+  <si>
+    <t>Half-year</t>
   </si>
 </sst>
 </file>
@@ -936,10 +936,10 @@
         <v>28</v>
       </c>
       <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
         <v>38</v>
-      </c>
-      <c r="C1" t="s">
-        <v>39</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
@@ -989,10 +989,10 @@
         <v>29</v>
       </c>
       <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D2" s="1">
         <v>2025</v>
@@ -1001,13 +1001,13 @@
         <v>35</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I2" s="1">
         <v>1</v>
@@ -1030,10 +1030,10 @@
         <v>29</v>
       </c>
       <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D3" s="1">
         <v>2025</v>
@@ -1042,13 +1042,13 @@
         <v>35</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I3" s="1">
         <v>2</v>
@@ -1112,10 +1112,10 @@
         <v>28</v>
       </c>
       <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
         <v>38</v>
-      </c>
-      <c r="C1" t="s">
-        <v>39</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -1189,10 +1189,10 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D2" s="1">
         <v>2025</v>
@@ -1201,13 +1201,13 @@
         <v>35</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I2" s="1">
         <v>1</v>
@@ -1245,10 +1245,10 @@
         <v>30</v>
       </c>
       <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D3" s="1">
         <v>2025</v>
@@ -1257,13 +1257,13 @@
         <v>35</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I3" s="1">
         <v>1</v>
@@ -1301,10 +1301,10 @@
         <v>30</v>
       </c>
       <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D4" s="1">
         <v>2025</v>
@@ -1313,13 +1313,13 @@
         <v>35</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I4" s="1">
         <v>1</v>
@@ -1357,10 +1357,10 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D5" s="1">
         <v>2025</v>
@@ -1369,13 +1369,13 @@
         <v>35</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I5" s="1">
         <v>1</v>
@@ -1413,10 +1413,10 @@
         <v>30</v>
       </c>
       <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D6" s="1">
         <v>2025</v>
@@ -1425,13 +1425,13 @@
         <v>35</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I6" s="1">
         <v>1</v>
@@ -1469,10 +1469,10 @@
         <v>30</v>
       </c>
       <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D7" s="1">
         <v>2025</v>
@@ -1481,13 +1481,13 @@
         <v>35</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I7" s="1">
         <v>1</v>
@@ -1525,10 +1525,10 @@
         <v>30</v>
       </c>
       <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D8" s="1">
         <v>2025</v>
@@ -1537,13 +1537,13 @@
         <v>35</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I8" s="1">
         <v>1</v>
@@ -1581,10 +1581,10 @@
         <v>30</v>
       </c>
       <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D9" s="1">
         <v>2025</v>
@@ -1593,13 +1593,13 @@
         <v>35</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I9" s="1">
         <v>1</v>
@@ -1637,10 +1637,10 @@
         <v>30</v>
       </c>
       <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D10" s="1">
         <v>2025</v>
@@ -1649,13 +1649,13 @@
         <v>35</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I10" s="1">
         <v>2</v>
@@ -1693,10 +1693,10 @@
         <v>30</v>
       </c>
       <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D11" s="1">
         <v>2025</v>
@@ -1705,13 +1705,13 @@
         <v>35</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I11" s="1">
         <v>2</v>
@@ -1749,10 +1749,10 @@
         <v>30</v>
       </c>
       <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D12" s="1">
         <v>2025</v>
@@ -1761,13 +1761,13 @@
         <v>35</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I12" s="1">
         <v>2</v>
@@ -1805,10 +1805,10 @@
         <v>30</v>
       </c>
       <c r="B13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D13" s="1">
         <v>2025</v>
@@ -1817,13 +1817,13 @@
         <v>35</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I13" s="1">
         <v>2</v>
@@ -1861,10 +1861,10 @@
         <v>30</v>
       </c>
       <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D14" s="1">
         <v>2025</v>
@@ -1873,13 +1873,13 @@
         <v>35</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I14" s="1">
         <v>2</v>
@@ -1917,10 +1917,10 @@
         <v>30</v>
       </c>
       <c r="B15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D15" s="1">
         <v>2025</v>
@@ -1929,13 +1929,13 @@
         <v>35</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I15" s="1">
         <v>2</v>
@@ -1973,10 +1973,10 @@
         <v>30</v>
       </c>
       <c r="B16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D16" s="1">
         <v>2025</v>
@@ -1985,13 +1985,13 @@
         <v>35</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I16" s="1">
         <v>2</v>
@@ -2029,10 +2029,10 @@
         <v>30</v>
       </c>
       <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="D17" s="1">
         <v>2025</v>
@@ -2041,13 +2041,13 @@
         <v>35</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I17" s="1">
         <v>2</v>
@@ -2259,18 +2259,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2292,6 +2292,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46D2B905-AB5A-461F-9589-9E2611C6FC90}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EF5FD55-8FE0-4218-9C8B-E5F035C6ADC7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -2307,14 +2315,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46D2B905-AB5A-461F-9589-9E2611C6FC90}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e0b220ce-5735-4468-91df-05cae5ff1fdc}" enabled="0" method="" siteId="{e0b220ce-5735-4468-91df-05cae5ff1fdc}" removed="1"/>

</xml_diff>